<commit_message>
feat: Correcciones de calculo
feat: Correcciones de calculo
</commit_message>
<xml_diff>
--- a/Analisis_Capacidad/Analisis_Capacidad.xlsx
+++ b/Analisis_Capacidad/Analisis_Capacidad.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\2026\SegundoSemestre2026\Modela\MYS2_Grupo2\Analisis_Capacidad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\2026\SegundoSemestre2026\Modela\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F600AD-E451-4125-9554-7015E2756F7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F47A593E-AB6A-4A82-BA68-3DA1DF9AAF3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -872,7 +872,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -933,6 +933,7 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1167,6 +1168,7 @@
     <xf numFmtId="164" fontId="0" fillId="14" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1180,11 +1182,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1490,10 +1487,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="102" t="s">
+      <c r="B1" s="104" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -1505,22 +1502,22 @@
       <c r="E1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="101" t="s">
+      <c r="F1" s="103" t="s">
         <v>137</v>
       </c>
-      <c r="G1" s="101" t="s">
+      <c r="G1" s="103" t="s">
         <v>138</v>
       </c>
-      <c r="H1" s="101" t="s">
+      <c r="H1" s="103" t="s">
         <v>153</v>
       </c>
-      <c r="I1" s="101" t="s">
+      <c r="I1" s="103" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="103"/>
-      <c r="B2" s="103"/>
+      <c r="A2" s="105"/>
+      <c r="B2" s="105"/>
       <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
@@ -1530,634 +1527,634 @@
       <c r="E2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="22">
+      <c r="A3" s="23">
         <v>1</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="25">
-        <v>2</v>
-      </c>
-      <c r="F3" s="26">
+      <c r="E3" s="26">
+        <v>2</v>
+      </c>
+      <c r="F3" s="27">
         <f>(1.98+2.2+2.42)/3</f>
         <v>2.1999999999999997</v>
       </c>
-      <c r="G3" s="26">
+      <c r="G3" s="27">
         <f>(1.98+2.2+2.42)/3</f>
         <v>2.1999999999999997</v>
       </c>
-      <c r="H3" s="26">
+      <c r="H3" s="27">
         <f t="shared" ref="H3:H8" si="0">F3*E3</f>
         <v>4.3999999999999995</v>
       </c>
-      <c r="I3" s="26">
+      <c r="I3" s="27">
         <f>G3*E3</f>
         <v>4.3999999999999995</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="22">
+      <c r="A4" s="23">
         <v>1</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="25">
+      <c r="E4" s="26">
         <v>3</v>
       </c>
-      <c r="F4" s="26">
+      <c r="F4" s="27">
         <f>(1.98+2.2+2.42)/3</f>
         <v>2.1999999999999997</v>
       </c>
-      <c r="G4" s="26">
+      <c r="G4" s="27">
         <f>(1.98+2.2+2.42)/3</f>
         <v>2.1999999999999997</v>
       </c>
-      <c r="H4" s="26">
+      <c r="H4" s="27">
         <f t="shared" si="0"/>
         <v>6.6</v>
       </c>
-      <c r="I4" s="26">
+      <c r="I4" s="27">
         <f>G4*E4</f>
         <v>6.6</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="22">
+      <c r="A5" s="23">
         <v>1</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="25">
-        <v>2</v>
-      </c>
-      <c r="F5" s="26">
+      <c r="E5" s="26">
+        <v>2</v>
+      </c>
+      <c r="F5" s="27">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="G5" s="26">
+      <c r="G5" s="27">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="H5" s="26">
+      <c r="H5" s="27">
         <f t="shared" si="0"/>
         <v>4.5999999999999988</v>
       </c>
-      <c r="I5" s="26">
+      <c r="I5" s="27">
         <f>G5*E5</f>
         <v>4.5999999999999988</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="27">
-        <v>2</v>
-      </c>
-      <c r="B6" s="28" t="s">
+      <c r="A6" s="28">
+        <v>2</v>
+      </c>
+      <c r="B6" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="30">
+      <c r="E6" s="31">
         <v>3</v>
       </c>
-      <c r="F6" s="31">
+      <c r="F6" s="32">
         <f>(10.3+12.1+13.4)/3</f>
         <v>11.933333333333332</v>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="32">
         <f>(10.3+12.1+13.4)/3</f>
         <v>11.933333333333332</v>
       </c>
-      <c r="H6" s="31">
+      <c r="H6" s="32">
         <f t="shared" si="0"/>
         <v>35.799999999999997</v>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="32">
         <f t="shared" ref="I6:I20" si="1">G6*E6</f>
         <v>35.799999999999997</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="27">
-        <v>2</v>
-      </c>
-      <c r="B7" s="28" t="s">
+      <c r="A7" s="28">
+        <v>2</v>
+      </c>
+      <c r="B7" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="30">
-        <v>2</v>
-      </c>
-      <c r="F7" s="31">
+      <c r="E7" s="31">
+        <v>2</v>
+      </c>
+      <c r="F7" s="32">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="G7" s="31">
+      <c r="G7" s="32">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="H7" s="31">
+      <c r="H7" s="32">
         <f t="shared" si="0"/>
         <v>3.4</v>
       </c>
-      <c r="I7" s="31">
+      <c r="I7" s="32">
         <f t="shared" si="1"/>
         <v>3.4</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="32">
+      <c r="A8" s="33">
         <v>3</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="35">
-        <v>2</v>
-      </c>
-      <c r="F8" s="36">
+      <c r="E8" s="36">
+        <v>2</v>
+      </c>
+      <c r="F8" s="37">
         <f>(1.62+1.8+1.98)/3</f>
         <v>1.8</v>
       </c>
-      <c r="G8" s="36">
+      <c r="G8" s="37">
         <f>(1+1.2+1.45)/3</f>
         <v>1.2166666666666668</v>
       </c>
-      <c r="H8" s="36">
+      <c r="H8" s="37">
         <f t="shared" si="0"/>
         <v>3.6</v>
       </c>
-      <c r="I8" s="36">
+      <c r="I8" s="37">
         <f>G8*E8</f>
         <v>2.4333333333333336</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="37">
+      <c r="A9" s="38">
         <v>4</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="39" t="s">
+      <c r="C9" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="39" t="s">
+      <c r="D9" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="40">
+      <c r="E9" s="41">
         <v>3</v>
       </c>
-      <c r="F9" s="41">
+      <c r="F9" s="42">
         <f>(1.8+2+2.2)/3</f>
         <v>2</v>
       </c>
-      <c r="G9" s="41">
+      <c r="G9" s="42">
         <f>(1.8+2+2.2)/3</f>
         <v>2</v>
       </c>
-      <c r="H9" s="41">
+      <c r="H9" s="42">
         <f t="shared" ref="H9:H21" si="2">F9*E9</f>
         <v>6</v>
       </c>
-      <c r="I9" s="41">
+      <c r="I9" s="42">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="37">
+      <c r="A10" s="38">
         <v>4</v>
       </c>
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="39" t="s">
+      <c r="D10" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="40">
-        <v>2</v>
-      </c>
-      <c r="F10" s="41">
+      <c r="E10" s="41">
+        <v>2</v>
+      </c>
+      <c r="F10" s="42">
         <f>(16+18+19)/3</f>
         <v>17.666666666666668</v>
       </c>
-      <c r="G10" s="41">
+      <c r="G10" s="42">
         <f>(14+16+18)/3</f>
         <v>16</v>
       </c>
-      <c r="H10" s="41">
+      <c r="H10" s="42">
         <f t="shared" si="2"/>
         <v>35.333333333333336</v>
       </c>
-      <c r="I10" s="41">
+      <c r="I10" s="42">
         <f t="shared" si="1"/>
         <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="37">
+      <c r="A11" s="38">
         <v>4</v>
       </c>
-      <c r="B11" s="38" t="s">
+      <c r="B11" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="39" t="s">
+      <c r="C11" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="D11" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="40">
-        <v>2</v>
-      </c>
-      <c r="F11" s="41">
+      <c r="E11" s="41">
+        <v>2</v>
+      </c>
+      <c r="F11" s="42">
         <f>(1.89+2.1+2.31)/3</f>
         <v>2.1</v>
       </c>
-      <c r="G11" s="41">
+      <c r="G11" s="42">
         <f>(1.89+2.1+2.31)/3</f>
         <v>2.1</v>
       </c>
-      <c r="H11" s="41">
+      <c r="H11" s="42">
         <f t="shared" si="2"/>
         <v>4.2</v>
       </c>
-      <c r="I11" s="41">
+      <c r="I11" s="42">
         <f t="shared" si="1"/>
         <v>4.2</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="42">
+      <c r="A12" s="43">
         <v>5</v>
       </c>
-      <c r="B12" s="43" t="s">
+      <c r="B12" s="44" t="s">
         <v>132</v>
       </c>
-      <c r="C12" s="44" t="s">
+      <c r="C12" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="44" t="s">
+      <c r="D12" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="45">
-        <v>2</v>
-      </c>
-      <c r="F12" s="46">
+      <c r="E12" s="46">
+        <v>2</v>
+      </c>
+      <c r="F12" s="47">
         <f>(2.34+2.6+2.86)/3</f>
         <v>2.5999999999999996</v>
       </c>
-      <c r="G12" s="46">
+      <c r="G12" s="47">
         <f>(2.34+2.6+2.86)/3</f>
         <v>2.5999999999999996</v>
       </c>
-      <c r="H12" s="46">
+      <c r="H12" s="47">
         <f t="shared" si="2"/>
         <v>5.1999999999999993</v>
       </c>
-      <c r="I12" s="46">
+      <c r="I12" s="47">
         <f t="shared" si="1"/>
         <v>5.1999999999999993</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="47">
+      <c r="A13" s="48">
         <v>6</v>
       </c>
-      <c r="B13" s="48" t="s">
+      <c r="B13" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="49" t="s">
+      <c r="C13" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="49" t="s">
+      <c r="D13" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="50">
+      <c r="E13" s="51">
         <v>4</v>
       </c>
-      <c r="F13" s="51">
+      <c r="F13" s="52">
         <f>(9+10+11)/3</f>
         <v>10</v>
       </c>
-      <c r="G13" s="51">
+      <c r="G13" s="52">
         <f>(9+11+12)/3</f>
         <v>10.666666666666666</v>
       </c>
-      <c r="H13" s="51">
+      <c r="H13" s="52">
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="I13" s="51">
+      <c r="I13" s="52">
         <f>G13*E13</f>
         <v>42.666666666666664</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="47">
+      <c r="A14" s="48">
         <v>6</v>
       </c>
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="49" t="s">
+      <c r="C14" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="49" t="s">
+      <c r="D14" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="50">
-        <v>2</v>
-      </c>
-      <c r="F14" s="51">
+      <c r="E14" s="51">
+        <v>2</v>
+      </c>
+      <c r="F14" s="52">
         <f>(1.71+1.9+2.09)/3</f>
         <v>1.8999999999999997</v>
       </c>
-      <c r="G14" s="51">
+      <c r="G14" s="52">
         <f>(1.71+1.9+2.09)/3</f>
         <v>1.8999999999999997</v>
       </c>
-      <c r="H14" s="51">
+      <c r="H14" s="52">
         <f t="shared" si="2"/>
         <v>3.7999999999999994</v>
       </c>
-      <c r="I14" s="51">
+      <c r="I14" s="52">
         <f t="shared" si="1"/>
         <v>3.7999999999999994</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="52">
+      <c r="A15" s="53">
         <v>7</v>
       </c>
-      <c r="B15" s="53" t="s">
+      <c r="B15" s="54" t="s">
         <v>133</v>
       </c>
-      <c r="C15" s="54" t="s">
+      <c r="C15" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="54" t="s">
+      <c r="D15" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="55">
+      <c r="E15" s="56">
         <v>5</v>
       </c>
-      <c r="F15" s="56">
+      <c r="F15" s="57">
         <f>(1.35+1.5+1.65)/3</f>
         <v>1.5</v>
       </c>
-      <c r="G15" s="56">
+      <c r="G15" s="57">
         <f>(1.35+1.5+1.65)/3</f>
         <v>1.5</v>
       </c>
-      <c r="H15" s="56">
+      <c r="H15" s="57">
         <f t="shared" si="2"/>
         <v>7.5</v>
       </c>
-      <c r="I15" s="56">
+      <c r="I15" s="57">
         <f t="shared" si="1"/>
         <v>7.5</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="52">
+      <c r="A16" s="53">
         <v>7</v>
       </c>
-      <c r="B16" s="53" t="s">
+      <c r="B16" s="54" t="s">
         <v>136</v>
       </c>
-      <c r="C16" s="54" t="s">
+      <c r="C16" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="54" t="s">
+      <c r="D16" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="55">
-        <v>2</v>
-      </c>
-      <c r="F16" s="56">
+      <c r="E16" s="56">
+        <v>2</v>
+      </c>
+      <c r="F16" s="57">
         <f>(5+6.5+7.2)/3</f>
         <v>6.2333333333333334</v>
       </c>
-      <c r="G16" s="56">
+      <c r="G16" s="57">
         <f>(5+6.5+7.2)/3</f>
         <v>6.2333333333333334</v>
       </c>
-      <c r="H16" s="56">
+      <c r="H16" s="57">
         <f t="shared" si="2"/>
         <v>12.466666666666667</v>
       </c>
-      <c r="I16" s="56">
+      <c r="I16" s="57">
         <f t="shared" si="1"/>
         <v>12.466666666666667</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="78">
+      <c r="A17" s="79">
         <v>8</v>
       </c>
-      <c r="B17" s="79" t="s">
+      <c r="B17" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="80" t="s">
+      <c r="C17" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="80" t="s">
+      <c r="D17" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="81">
-        <v>2</v>
-      </c>
-      <c r="F17" s="82">
+      <c r="E17" s="82">
+        <v>2</v>
+      </c>
+      <c r="F17" s="83">
         <f>(0.72+0.8+0.88)/3</f>
         <v>0.79999999999999993</v>
       </c>
-      <c r="G17" s="82">
+      <c r="G17" s="83">
         <f>(0.72+0.8+0.88)/3</f>
         <v>0.79999999999999993</v>
       </c>
-      <c r="H17" s="82">
+      <c r="H17" s="83">
         <f>F17*E17</f>
         <v>1.5999999999999999</v>
       </c>
-      <c r="I17" s="82">
+      <c r="I17" s="83">
         <f t="shared" si="1"/>
         <v>1.5999999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="57">
+      <c r="A18" s="58">
         <v>9</v>
       </c>
-      <c r="B18" s="58" t="s">
+      <c r="B18" s="59" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="59" t="s">
+      <c r="C18" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="D18" s="59" t="s">
+      <c r="D18" s="60" t="s">
         <v>36</v>
       </c>
-      <c r="E18" s="60">
+      <c r="E18" s="61">
         <v>3</v>
       </c>
-      <c r="F18" s="61">
+      <c r="F18" s="62">
         <f>(21+25.2+27)/3</f>
         <v>24.400000000000002</v>
       </c>
-      <c r="G18" s="61">
+      <c r="G18" s="62">
         <f>(9+11.5+14)/3</f>
         <v>11.5</v>
       </c>
-      <c r="H18" s="61">
+      <c r="H18" s="62">
         <f t="shared" si="2"/>
         <v>73.2</v>
       </c>
-      <c r="I18" s="61">
+      <c r="I18" s="62">
         <f t="shared" si="1"/>
         <v>34.5</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="68">
+      <c r="A19" s="69">
         <v>10</v>
       </c>
-      <c r="B19" s="69" t="s">
+      <c r="B19" s="70" t="s">
         <v>134</v>
       </c>
-      <c r="C19" s="70" t="s">
+      <c r="C19" s="71" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="70" t="s">
+      <c r="D19" s="71" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="71">
-        <v>2</v>
-      </c>
-      <c r="F19" s="72">
+      <c r="E19" s="72">
+        <v>2</v>
+      </c>
+      <c r="F19" s="73">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="G19" s="72">
+      <c r="G19" s="73">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="H19" s="72">
+      <c r="H19" s="73">
         <f>F19*E19</f>
         <v>3.4</v>
       </c>
-      <c r="I19" s="72">
+      <c r="I19" s="73">
         <f>G19*E19</f>
         <v>3.4</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="68">
+      <c r="A20" s="69">
         <v>10</v>
       </c>
-      <c r="B20" s="69" t="s">
+      <c r="B20" s="70" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="70" t="s">
+      <c r="C20" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="70" t="s">
+      <c r="D20" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="E20" s="71">
-        <v>2</v>
-      </c>
-      <c r="F20" s="72">
+      <c r="E20" s="72">
+        <v>2</v>
+      </c>
+      <c r="F20" s="73">
         <f>(0.72+0.8+0.88)/3</f>
         <v>0.79999999999999993</v>
       </c>
-      <c r="G20" s="72">
+      <c r="G20" s="73">
         <f>(0.72+0.8+0.88)/3</f>
         <v>0.79999999999999993</v>
       </c>
-      <c r="H20" s="72">
+      <c r="H20" s="73">
         <f t="shared" si="2"/>
         <v>1.5999999999999999</v>
       </c>
-      <c r="I20" s="72">
+      <c r="I20" s="73">
         <f t="shared" si="1"/>
         <v>1.5999999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="73">
+      <c r="A21" s="74">
         <v>11</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="B21" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="C21" s="75" t="s">
+      <c r="C21" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="75" t="s">
+      <c r="D21" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="E21" s="76">
+      <c r="E21" s="77">
         <v>4</v>
       </c>
-      <c r="F21" s="77">
+      <c r="F21" s="78">
         <f>(0.45+0.5+0.55)/3</f>
         <v>0.5</v>
       </c>
-      <c r="G21" s="77">
+      <c r="G21" s="78">
         <f>(0.45+0.5+0.55)/3</f>
         <v>0.5</v>
       </c>
-      <c r="H21" s="77">
+      <c r="H21" s="78">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="I21" s="77">
+      <c r="I21" s="78">
         <f>G21*E21</f>
         <v>2</v>
       </c>
@@ -2435,16 +2432,16 @@
       <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="101" t="s">
+      <c r="F1" s="103" t="s">
         <v>137</v>
       </c>
-      <c r="G1" s="101" t="s">
+      <c r="G1" s="103" t="s">
         <v>138</v>
       </c>
-      <c r="H1" s="101" t="s">
+      <c r="H1" s="103" t="s">
         <v>153</v>
       </c>
-      <c r="I1" s="101" t="s">
+      <c r="I1" s="103" t="s">
         <v>154</v>
       </c>
     </row>
@@ -2460,667 +2457,667 @@
       <c r="E2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="22">
+      <c r="A3" s="23">
         <v>1</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="65" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="E3" s="65">
-        <v>2</v>
-      </c>
-      <c r="F3" s="26">
+      <c r="E3" s="66">
+        <v>2</v>
+      </c>
+      <c r="F3" s="27">
         <f>(1.98+2.2+2.42)/3</f>
         <v>2.1999999999999997</v>
       </c>
-      <c r="G3" s="26">
+      <c r="G3" s="27">
         <f>(2.1+2.8+3.17)/3</f>
         <v>2.69</v>
       </c>
-      <c r="H3" s="26">
+      <c r="H3" s="27">
         <f>F3*E3</f>
         <v>4.3999999999999995</v>
       </c>
-      <c r="I3" s="26">
+      <c r="I3" s="27">
         <f>G3*E3</f>
         <v>5.38</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="22">
+      <c r="A4" s="23">
         <v>1</v>
       </c>
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="65" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="65">
+      <c r="E4" s="66">
         <v>3</v>
       </c>
-      <c r="F4" s="26">
+      <c r="F4" s="27">
         <f>(5+6.5+7.2)/3</f>
         <v>6.2333333333333334</v>
       </c>
-      <c r="G4" s="26">
+      <c r="G4" s="27">
         <f>(4.3+5.5+6.8)/3</f>
         <v>5.5333333333333341</v>
       </c>
-      <c r="H4" s="26">
+      <c r="H4" s="27">
         <f t="shared" ref="H4:H22" si="0">F4*E4</f>
         <v>18.7</v>
       </c>
-      <c r="I4" s="26">
+      <c r="I4" s="27">
         <f t="shared" ref="I4:I22" si="1">G4*E4</f>
         <v>16.600000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27">
-        <v>2</v>
-      </c>
-      <c r="B5" s="66" t="s">
+      <c r="A5" s="28">
+        <v>2</v>
+      </c>
+      <c r="B5" s="67" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="67">
-        <v>2</v>
-      </c>
-      <c r="F5" s="31">
+      <c r="E5" s="68">
+        <v>2</v>
+      </c>
+      <c r="F5" s="32">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="G5" s="31">
+      <c r="G5" s="32">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="H5" s="31">
+      <c r="H5" s="32">
         <f t="shared" si="0"/>
         <v>4.5999999999999988</v>
       </c>
-      <c r="I5" s="31">
+      <c r="I5" s="32">
         <f t="shared" si="1"/>
         <v>4.5999999999999988</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="27">
-        <v>2</v>
-      </c>
-      <c r="B6" s="66" t="s">
+      <c r="A6" s="28">
+        <v>2</v>
+      </c>
+      <c r="B6" s="67" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="67">
-        <v>2</v>
-      </c>
-      <c r="F6" s="31">
+      <c r="E6" s="68">
+        <v>2</v>
+      </c>
+      <c r="F6" s="32">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="32">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="H6" s="31">
+      <c r="H6" s="32">
         <f t="shared" si="0"/>
         <v>4.5999999999999988</v>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="32">
         <f t="shared" si="1"/>
         <v>4.5999999999999988</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="27">
-        <v>2</v>
-      </c>
-      <c r="B7" s="66" t="s">
+      <c r="A7" s="28">
+        <v>2</v>
+      </c>
+      <c r="B7" s="67" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="E7" s="67">
+      <c r="E7" s="68">
         <v>3</v>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="32">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="G7" s="31">
+      <c r="G7" s="32">
         <f>(1.4+1.7+1.8)/3</f>
         <v>1.6333333333333331</v>
       </c>
-      <c r="H7" s="31">
+      <c r="H7" s="32">
         <f t="shared" si="0"/>
         <v>5.0999999999999996</v>
       </c>
-      <c r="I7" s="31">
+      <c r="I7" s="32">
         <f t="shared" si="1"/>
         <v>4.8999999999999995</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="32">
+      <c r="A8" s="33">
         <v>3</v>
       </c>
-      <c r="B8" s="62" t="s">
+      <c r="B8" s="63" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="63">
-        <v>2</v>
-      </c>
-      <c r="F8" s="36">
+      <c r="E8" s="64">
+        <v>2</v>
+      </c>
+      <c r="F8" s="37">
         <f>(16.2+18+19.8)/3</f>
         <v>18</v>
       </c>
-      <c r="G8" s="36">
+      <c r="G8" s="37">
         <f>(16.2+18+19.8)/3</f>
         <v>18</v>
       </c>
-      <c r="H8" s="36">
+      <c r="H8" s="37">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="I8" s="36">
+      <c r="I8" s="37">
         <f t="shared" si="1"/>
         <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="32">
+      <c r="A9" s="33">
         <v>3</v>
       </c>
-      <c r="B9" s="62" t="s">
+      <c r="B9" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="D9" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="63">
+      <c r="E9" s="64">
         <v>3</v>
       </c>
-      <c r="F9" s="36">
+      <c r="F9" s="37">
         <f>(1.8+2+2.2)/3</f>
         <v>2</v>
       </c>
-      <c r="G9" s="36">
+      <c r="G9" s="37">
         <f>(1.8+2+2.2)/3</f>
         <v>2</v>
       </c>
-      <c r="H9" s="36">
+      <c r="H9" s="37">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="I9" s="36">
+      <c r="I9" s="37">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="37">
+      <c r="A10" s="38">
         <v>4</v>
       </c>
-      <c r="B10" s="83" t="s">
+      <c r="B10" s="84" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="39" t="s">
+      <c r="D10" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="84">
-        <v>2</v>
-      </c>
-      <c r="F10" s="41">
+      <c r="E10" s="85">
+        <v>2</v>
+      </c>
+      <c r="F10" s="42">
         <f>(12+13.5+13.9)/3</f>
         <v>13.133333333333333</v>
       </c>
-      <c r="G10" s="41">
+      <c r="G10" s="42">
         <f>(9+11.2+13.6)/3</f>
         <v>11.266666666666666</v>
       </c>
-      <c r="H10" s="41">
+      <c r="H10" s="42">
         <f t="shared" si="0"/>
         <v>26.266666666666666</v>
       </c>
-      <c r="I10" s="41">
+      <c r="I10" s="42">
         <f t="shared" si="1"/>
         <v>22.533333333333331</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="37">
+      <c r="A11" s="38">
         <v>4</v>
       </c>
-      <c r="B11" s="83" t="s">
+      <c r="B11" s="84" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="39" t="s">
+      <c r="C11" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="D11" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="84">
-        <v>2</v>
-      </c>
-      <c r="F11" s="41">
+      <c r="E11" s="85">
+        <v>2</v>
+      </c>
+      <c r="F11" s="42">
         <f>(1.89+2.1+2.31)/3</f>
         <v>2.1</v>
       </c>
-      <c r="G11" s="41">
+      <c r="G11" s="42">
         <f>(1.89+2.1+2.31)/3</f>
         <v>2.1</v>
       </c>
-      <c r="H11" s="41">
+      <c r="H11" s="42">
         <f t="shared" si="0"/>
         <v>4.2</v>
       </c>
-      <c r="I11" s="41">
+      <c r="I11" s="42">
         <f t="shared" si="1"/>
         <v>4.2</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="42">
+      <c r="A12" s="43">
         <v>5</v>
       </c>
-      <c r="B12" s="85" t="s">
+      <c r="B12" s="86" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="44" t="s">
+      <c r="C12" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="44" t="s">
+      <c r="D12" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="E12" s="86">
+      <c r="E12" s="87">
         <v>3</v>
       </c>
-      <c r="F12" s="46">
+      <c r="F12" s="47">
         <f>(8.4+10.1+12.6)/3</f>
         <v>10.366666666666667</v>
       </c>
-      <c r="G12" s="46">
+      <c r="G12" s="47">
         <f>(8.4+10.1+12.6)/3</f>
         <v>10.366666666666667</v>
       </c>
-      <c r="H12" s="46">
+      <c r="H12" s="47">
         <f t="shared" si="0"/>
         <v>31.1</v>
       </c>
-      <c r="I12" s="46">
+      <c r="I12" s="47">
         <f t="shared" si="1"/>
         <v>31.1</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="42">
+      <c r="A13" s="43">
         <v>5</v>
       </c>
-      <c r="B13" s="85" t="s">
+      <c r="B13" s="86" t="s">
         <v>56</v>
       </c>
-      <c r="C13" s="44" t="s">
+      <c r="C13" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="D13" s="44" t="s">
+      <c r="D13" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="E13" s="86">
-        <v>2</v>
-      </c>
-      <c r="F13" s="46">
+      <c r="E13" s="87">
+        <v>2</v>
+      </c>
+      <c r="F13" s="47">
         <f>(0.9+1+1.1)/3</f>
         <v>1</v>
       </c>
-      <c r="G13" s="46">
+      <c r="G13" s="47">
         <f>(1+2.2+4.1)/3</f>
         <v>2.4333333333333331</v>
       </c>
-      <c r="H13" s="46">
+      <c r="H13" s="47">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="I13" s="46">
+      <c r="I13" s="47">
         <f t="shared" si="1"/>
         <v>4.8666666666666663</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="47">
+      <c r="A14" s="48">
         <v>6</v>
       </c>
-      <c r="B14" s="87" t="s">
+      <c r="B14" s="88" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="49" t="s">
+      <c r="C14" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="D14" s="49" t="s">
+      <c r="D14" s="50" t="s">
         <v>61</v>
       </c>
-      <c r="E14" s="88">
+      <c r="E14" s="89">
         <v>3</v>
       </c>
-      <c r="F14" s="51">
+      <c r="F14" s="52">
         <f>(12+15+17)/3</f>
         <v>14.666666666666666</v>
       </c>
-      <c r="G14" s="51">
+      <c r="G14" s="52">
         <f>(13.2+15+17.5)/3</f>
         <v>15.233333333333334</v>
       </c>
-      <c r="H14" s="51">
+      <c r="H14" s="52">
         <f>F14*E14</f>
         <v>44</v>
       </c>
-      <c r="I14" s="51">
+      <c r="I14" s="52">
         <f>G14*E14</f>
         <v>45.7</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="47">
+      <c r="A15" s="48">
         <v>6</v>
       </c>
-      <c r="B15" s="87" t="s">
+      <c r="B15" s="88" t="s">
         <v>62</v>
       </c>
-      <c r="C15" s="49" t="s">
+      <c r="C15" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="49" t="s">
+      <c r="D15" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="88">
-        <v>2</v>
-      </c>
-      <c r="F15" s="51">
+      <c r="E15" s="89">
+        <v>2</v>
+      </c>
+      <c r="F15" s="52">
         <f>(1.35+1.5+1.65)/3</f>
         <v>1.5</v>
       </c>
-      <c r="G15" s="51">
+      <c r="G15" s="52">
         <f>(1.35+1.5+1.65)/3</f>
         <v>1.5</v>
       </c>
-      <c r="H15" s="51">
+      <c r="H15" s="52">
         <f>F15*E15</f>
         <v>3</v>
       </c>
-      <c r="I15" s="51">
+      <c r="I15" s="52">
         <f>G15*E15</f>
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="52">
+      <c r="A16" s="53">
         <v>7</v>
       </c>
-      <c r="B16" s="89" t="s">
+      <c r="B16" s="90" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="54" t="s">
+      <c r="C16" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="54" t="s">
+      <c r="D16" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="90">
+      <c r="E16" s="91">
         <v>4</v>
       </c>
-      <c r="F16" s="56">
+      <c r="F16" s="57">
         <f>(5+6.5+7.2)/3</f>
         <v>6.2333333333333334</v>
       </c>
-      <c r="G16" s="56">
+      <c r="G16" s="57">
         <f>(5+6.5+7.2)/3</f>
         <v>6.2333333333333334</v>
       </c>
-      <c r="H16" s="56">
+      <c r="H16" s="57">
         <f t="shared" si="0"/>
         <v>24.933333333333334</v>
       </c>
-      <c r="I16" s="56">
+      <c r="I16" s="57">
         <f t="shared" si="1"/>
         <v>24.933333333333334</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="78">
+      <c r="A17" s="79">
         <v>8</v>
       </c>
-      <c r="B17" s="91" t="s">
+      <c r="B17" s="92" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="80" t="s">
+      <c r="C17" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="80" t="s">
+      <c r="D17" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="92">
-        <v>2</v>
-      </c>
-      <c r="F17" s="82">
+      <c r="E17" s="93">
+        <v>2</v>
+      </c>
+      <c r="F17" s="83">
         <f>(0.72+0.8+0.88)/3</f>
         <v>0.79999999999999993</v>
       </c>
-      <c r="G17" s="82">
+      <c r="G17" s="83">
         <f>(0.72+0.8+0.88)/3</f>
         <v>0.79999999999999993</v>
       </c>
-      <c r="H17" s="82">
+      <c r="H17" s="83">
         <f t="shared" si="0"/>
         <v>1.5999999999999999</v>
       </c>
-      <c r="I17" s="82">
+      <c r="I17" s="83">
         <f t="shared" si="1"/>
         <v>1.5999999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="78">
+      <c r="A18" s="79">
         <v>8</v>
       </c>
-      <c r="B18" s="91" t="s">
+      <c r="B18" s="92" t="s">
         <v>56</v>
       </c>
-      <c r="C18" s="80" t="s">
+      <c r="C18" s="81" t="s">
         <v>64</v>
       </c>
-      <c r="D18" s="80" t="s">
+      <c r="D18" s="81" t="s">
         <v>64</v>
       </c>
-      <c r="E18" s="92">
+      <c r="E18" s="93">
         <v>4</v>
       </c>
-      <c r="F18" s="82">
+      <c r="F18" s="83">
         <f>(16+18+19.5)/3</f>
         <v>17.833333333333332</v>
       </c>
-      <c r="G18" s="82">
+      <c r="G18" s="83">
         <f>(16+18+19.5)/3</f>
         <v>17.833333333333332</v>
       </c>
-      <c r="H18" s="82">
+      <c r="H18" s="83">
         <f t="shared" si="0"/>
         <v>71.333333333333329</v>
       </c>
-      <c r="I18" s="82">
+      <c r="I18" s="83">
         <f t="shared" si="1"/>
         <v>71.333333333333329</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="57">
+      <c r="A19" s="58">
         <v>9</v>
       </c>
-      <c r="B19" s="93" t="s">
+      <c r="B19" s="94" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="59" t="s">
+      <c r="C19" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="59" t="s">
+      <c r="D19" s="60" t="s">
         <v>66</v>
       </c>
-      <c r="E19" s="94">
-        <v>2</v>
-      </c>
-      <c r="F19" s="61">
+      <c r="E19" s="95">
+        <v>2</v>
+      </c>
+      <c r="F19" s="62">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="G19" s="61">
+      <c r="G19" s="62">
         <f>(1.4+1.9+2.3)/3</f>
         <v>1.8666666666666665</v>
       </c>
-      <c r="H19" s="61">
+      <c r="H19" s="62">
         <f t="shared" si="0"/>
         <v>3.4</v>
       </c>
-      <c r="I19" s="61">
+      <c r="I19" s="62">
         <f t="shared" si="1"/>
         <v>3.7333333333333329</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="68">
+      <c r="A20" s="69">
         <v>10</v>
       </c>
-      <c r="B20" s="95" t="s">
+      <c r="B20" s="96" t="s">
         <v>67</v>
       </c>
-      <c r="C20" s="70" t="s">
+      <c r="C20" s="71" t="s">
         <v>68</v>
       </c>
-      <c r="D20" s="70" t="s">
+      <c r="D20" s="71" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="96">
+      <c r="E20" s="97">
         <v>3</v>
       </c>
-      <c r="F20" s="72">
+      <c r="F20" s="73">
         <f>(7+11+12.5)/3</f>
         <v>10.166666666666666</v>
       </c>
-      <c r="G20" s="72">
+      <c r="G20" s="73">
         <f>(7+11+12.5)/3</f>
         <v>10.166666666666666</v>
       </c>
-      <c r="H20" s="72">
+      <c r="H20" s="73">
         <f t="shared" si="0"/>
         <v>30.5</v>
       </c>
-      <c r="I20" s="72">
+      <c r="I20" s="73">
         <f t="shared" si="1"/>
         <v>30.5</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="73">
+      <c r="A21" s="74">
         <v>11</v>
       </c>
-      <c r="B21" s="97" t="s">
+      <c r="B21" s="98" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="75" t="s">
+      <c r="C21" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="75" t="s">
+      <c r="D21" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="E21" s="98">
+      <c r="E21" s="99">
         <v>1</v>
       </c>
-      <c r="F21" s="77">
+      <c r="F21" s="78">
         <f>(0.45+0.5+0.55)/3</f>
         <v>0.5</v>
       </c>
-      <c r="G21" s="77">
+      <c r="G21" s="78">
         <f>(0.45+0.5+0.55)/3</f>
         <v>0.5</v>
       </c>
-      <c r="H21" s="77">
+      <c r="H21" s="78">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="I21" s="77">
+      <c r="I21" s="78">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="73">
+      <c r="A22" s="74">
         <v>11</v>
       </c>
-      <c r="B22" s="97" t="s">
+      <c r="B22" s="98" t="s">
         <v>70</v>
       </c>
-      <c r="C22" s="75" t="s">
+      <c r="C22" s="76" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="75" t="s">
+      <c r="D22" s="76" t="s">
         <v>29</v>
       </c>
-      <c r="E22" s="98">
+      <c r="E22" s="99">
         <v>1</v>
       </c>
-      <c r="F22" s="99">
+      <c r="F22" s="100">
         <f>(1.71+1.9+2.09)/3</f>
         <v>1.8999999999999997</v>
       </c>
-      <c r="G22" s="99">
+      <c r="G22" s="100">
         <f>(1.71+1.9+2.09)/3</f>
         <v>1.8999999999999997</v>
       </c>
-      <c r="H22" s="77">
+      <c r="H22" s="78">
         <f t="shared" si="0"/>
         <v>1.8999999999999997</v>
       </c>
-      <c r="I22" s="77">
+      <c r="I22" s="78">
         <f t="shared" si="1"/>
         <v>1.8999999999999997</v>
       </c>
@@ -3385,10 +3382,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="102" t="s">
+      <c r="B1" s="104" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -3400,22 +3397,22 @@
       <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="101" t="s">
+      <c r="F1" s="103" t="s">
         <v>137</v>
       </c>
-      <c r="G1" s="101" t="s">
+      <c r="G1" s="103" t="s">
         <v>138</v>
       </c>
-      <c r="H1" s="101" t="s">
+      <c r="H1" s="103" t="s">
         <v>153</v>
       </c>
-      <c r="I1" s="101" t="s">
+      <c r="I1" s="103" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="103"/>
-      <c r="B2" s="103"/>
+      <c r="A2" s="105"/>
+      <c r="B2" s="105"/>
       <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
@@ -3425,634 +3422,634 @@
       <c r="E2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="22">
+      <c r="A3" s="23">
         <v>1</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="E3" s="65">
-        <v>2</v>
-      </c>
-      <c r="F3" s="26">
+      <c r="E3" s="66">
+        <v>2</v>
+      </c>
+      <c r="F3" s="27">
         <f>(1.98+2.2+2.42)/3</f>
         <v>2.1999999999999997</v>
       </c>
-      <c r="G3" s="26">
+      <c r="G3" s="27">
         <f>(1.33+2.25+2.98)/3</f>
         <v>2.186666666666667</v>
       </c>
-      <c r="H3" s="26">
+      <c r="H3" s="27">
         <f>F3*E3</f>
         <v>4.3999999999999995</v>
       </c>
-      <c r="I3" s="26">
+      <c r="I3" s="27">
         <f>G3*E3</f>
         <v>4.373333333333334</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="22">
+      <c r="A4" s="23">
         <v>1</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="E4" s="65">
+      <c r="E4" s="66">
         <v>3</v>
       </c>
-      <c r="F4" s="26">
+      <c r="F4" s="27">
         <f>(5+6.5+7.2)/3</f>
         <v>6.2333333333333334</v>
       </c>
-      <c r="G4" s="26">
+      <c r="G4" s="27">
         <f>(4.2+5.4+6.23)/3</f>
         <v>5.2766666666666673</v>
       </c>
-      <c r="H4" s="26">
+      <c r="H4" s="27">
         <f t="shared" ref="H4:H21" si="0">F4*E4</f>
         <v>18.7</v>
       </c>
-      <c r="I4" s="26">
+      <c r="I4" s="27">
         <f t="shared" ref="I4:I21" si="1">G4*E4</f>
         <v>15.830000000000002</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="22">
+      <c r="A5" s="23">
         <v>1</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="24" t="s">
         <v>129</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="65">
-        <v>2</v>
-      </c>
-      <c r="F5" s="26">
+      <c r="E5" s="66">
+        <v>2</v>
+      </c>
+      <c r="F5" s="27">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="G5" s="26">
+      <c r="G5" s="27">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="H5" s="26">
+      <c r="H5" s="27">
         <f t="shared" si="0"/>
         <v>4.5999999999999988</v>
       </c>
-      <c r="I5" s="26">
+      <c r="I5" s="27">
         <f t="shared" si="1"/>
         <v>4.5999999999999988</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="27">
-        <v>2</v>
-      </c>
-      <c r="B6" s="28" t="s">
+      <c r="A6" s="28">
+        <v>2</v>
+      </c>
+      <c r="B6" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="67">
-        <v>2</v>
-      </c>
-      <c r="F6" s="31">
+      <c r="E6" s="68">
+        <v>2</v>
+      </c>
+      <c r="F6" s="32">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="32">
         <f>(2.1+2.45+2.58)/3</f>
         <v>2.3766666666666669</v>
       </c>
-      <c r="H6" s="31">
+      <c r="H6" s="32">
         <f t="shared" si="0"/>
         <v>4.5999999999999988</v>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="32">
         <f t="shared" si="1"/>
         <v>4.7533333333333339</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="27">
-        <v>2</v>
-      </c>
-      <c r="B7" s="28" t="s">
+      <c r="A7" s="28">
+        <v>2</v>
+      </c>
+      <c r="B7" s="29" t="s">
         <v>76</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="67">
-        <v>2</v>
-      </c>
-      <c r="F7" s="31">
+      <c r="E7" s="68">
+        <v>2</v>
+      </c>
+      <c r="F7" s="32">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="G7" s="31">
+      <c r="G7" s="32">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="H7" s="31">
+      <c r="H7" s="32">
         <f t="shared" si="0"/>
         <v>3.4</v>
       </c>
-      <c r="I7" s="31">
+      <c r="I7" s="32">
         <f t="shared" si="1"/>
         <v>3.4</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="32">
+      <c r="A8" s="33">
         <v>3</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="E8" s="63">
-        <v>2</v>
-      </c>
-      <c r="F8" s="36">
+      <c r="E8" s="64">
+        <v>2</v>
+      </c>
+      <c r="F8" s="37">
         <f>(1.62+1.8+1.98)/3</f>
         <v>1.8</v>
       </c>
-      <c r="G8" s="36">
-        <f>(1.62+1.8+1.98)/3</f>
-        <v>1.8</v>
-      </c>
-      <c r="H8" s="36">
-        <f t="shared" si="0"/>
+      <c r="G8" s="37">
+        <f>(1.2+1.34+1.6)/3</f>
+        <v>1.3800000000000001</v>
+      </c>
+      <c r="H8" s="37">
+        <f>F8*E8</f>
         <v>3.6</v>
       </c>
-      <c r="I8" s="36">
-        <f t="shared" si="1"/>
-        <v>3.6</v>
+      <c r="I8" s="37">
+        <f t="shared" si="1"/>
+        <v>2.7600000000000002</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="37">
+      <c r="A9" s="38">
         <v>4</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="39" t="s">
         <v>78</v>
       </c>
-      <c r="C9" s="39" t="s">
+      <c r="C9" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="39" t="s">
+      <c r="D9" s="40" t="s">
         <v>79</v>
       </c>
-      <c r="E9" s="84">
+      <c r="E9" s="85">
         <v>3</v>
       </c>
-      <c r="F9" s="41">
+      <c r="F9" s="42">
         <f>(1.8+2+2.2)/3</f>
         <v>2</v>
       </c>
-      <c r="G9" s="41">
+      <c r="G9" s="42">
         <f>(1.2+3.3+4.1)/3</f>
         <v>2.8666666666666667</v>
       </c>
-      <c r="H9" s="41">
+      <c r="H9" s="42">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="I9" s="41">
+      <c r="I9" s="42">
         <f t="shared" si="1"/>
         <v>8.6</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="37">
+      <c r="A10" s="38">
         <v>4</v>
       </c>
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="39" t="s">
         <v>80</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="40" t="s">
         <v>81</v>
       </c>
-      <c r="D10" s="39" t="s">
+      <c r="D10" s="40" t="s">
         <v>82</v>
       </c>
-      <c r="E10" s="84">
-        <v>2</v>
-      </c>
-      <c r="F10" s="41">
+      <c r="E10" s="85">
+        <v>2</v>
+      </c>
+      <c r="F10" s="42">
         <f>(12+13.4+14.2)/3</f>
         <v>13.199999999999998</v>
       </c>
-      <c r="G10" s="41">
+      <c r="G10" s="42">
         <f>(15+16.4+17)/3</f>
         <v>16.133333333333333</v>
       </c>
-      <c r="H10" s="41">
+      <c r="H10" s="42">
         <f t="shared" si="0"/>
         <v>26.399999999999995</v>
       </c>
-      <c r="I10" s="41">
+      <c r="I10" s="42">
         <f>G10*E10</f>
         <v>32.266666666666666</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="37">
+      <c r="A11" s="38">
         <v>4</v>
       </c>
-      <c r="B11" s="38" t="s">
+      <c r="B11" s="39" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="39" t="s">
+      <c r="C11" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="D11" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="84">
-        <v>2</v>
-      </c>
-      <c r="F11" s="41">
+      <c r="E11" s="85">
+        <v>2</v>
+      </c>
+      <c r="F11" s="42">
         <f>(1.89+2.1+2.31)/3</f>
         <v>2.1</v>
       </c>
-      <c r="G11" s="41">
+      <c r="G11" s="42">
         <f>(1.89+2.1+2.31)/3</f>
         <v>2.1</v>
       </c>
-      <c r="H11" s="41">
+      <c r="H11" s="42">
         <f t="shared" si="0"/>
         <v>4.2</v>
       </c>
-      <c r="I11" s="41">
+      <c r="I11" s="42">
         <f t="shared" si="1"/>
         <v>4.2</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="42">
+      <c r="A12" s="43">
         <v>5</v>
       </c>
-      <c r="B12" s="43" t="s">
+      <c r="B12" s="44" t="s">
         <v>84</v>
       </c>
-      <c r="C12" s="44" t="s">
+      <c r="C12" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="44" t="s">
+      <c r="D12" s="45" t="s">
         <v>85</v>
       </c>
-      <c r="E12" s="86">
-        <v>2</v>
-      </c>
-      <c r="F12" s="46">
+      <c r="E12" s="87">
+        <v>2</v>
+      </c>
+      <c r="F12" s="47">
         <f>(2.34+2.6+2.86)/3</f>
         <v>2.5999999999999996</v>
       </c>
-      <c r="G12" s="46">
+      <c r="G12" s="47">
         <f>(2.44+2.65+3.6)/3</f>
         <v>2.8966666666666665</v>
       </c>
-      <c r="H12" s="46">
+      <c r="H12" s="47">
         <f t="shared" si="0"/>
         <v>5.1999999999999993</v>
       </c>
-      <c r="I12" s="46">
+      <c r="I12" s="47">
         <f t="shared" si="1"/>
         <v>5.793333333333333</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="47">
+      <c r="A13" s="48">
         <v>6</v>
       </c>
-      <c r="B13" s="48" t="s">
+      <c r="B13" s="49" t="s">
         <v>80</v>
       </c>
-      <c r="C13" s="49" t="s">
+      <c r="C13" s="50" t="s">
         <v>86</v>
       </c>
-      <c r="D13" s="49" t="s">
+      <c r="D13" s="50" t="s">
         <v>87</v>
       </c>
-      <c r="E13" s="88">
+      <c r="E13" s="89">
         <v>5</v>
       </c>
-      <c r="F13" s="51">
+      <c r="F13" s="52">
         <f>(4+6.3+7.1)/3</f>
         <v>5.8</v>
       </c>
-      <c r="G13" s="51">
+      <c r="G13" s="52">
         <f>(3.3+5.4+6.1)/3</f>
         <v>4.9333333333333327</v>
       </c>
-      <c r="H13" s="51">
+      <c r="H13" s="52">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="I13" s="51">
+      <c r="I13" s="52">
         <f t="shared" si="1"/>
         <v>24.666666666666664</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="47">
+      <c r="A14" s="48">
         <v>6</v>
       </c>
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="49" t="s">
         <v>83</v>
       </c>
-      <c r="C14" s="49" t="s">
+      <c r="C14" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="D14" s="49" t="s">
+      <c r="D14" s="50" t="s">
         <v>88</v>
       </c>
-      <c r="E14" s="88">
-        <v>2</v>
-      </c>
-      <c r="F14" s="51">
+      <c r="E14" s="89">
+        <v>2</v>
+      </c>
+      <c r="F14" s="52">
         <f>(12+15+17)/3</f>
         <v>14.666666666666666</v>
       </c>
-      <c r="G14" s="51">
+      <c r="G14" s="52">
         <f>(10+12+15)/3</f>
         <v>12.333333333333334</v>
       </c>
-      <c r="H14" s="51">
+      <c r="H14" s="52">
         <f t="shared" si="0"/>
         <v>29.333333333333332</v>
       </c>
-      <c r="I14" s="51">
+      <c r="I14" s="52">
         <f t="shared" si="1"/>
         <v>24.666666666666668</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="52">
+      <c r="A15" s="53">
         <v>7</v>
       </c>
-      <c r="B15" s="53" t="s">
+      <c r="B15" s="54" t="s">
         <v>89</v>
       </c>
-      <c r="C15" s="54" t="s">
+      <c r="C15" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="54" t="s">
+      <c r="D15" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="90">
+      <c r="E15" s="91">
         <v>4</v>
       </c>
-      <c r="F15" s="56">
+      <c r="F15" s="57">
         <f>(1.35+1.5+1.65)/3</f>
         <v>1.5</v>
       </c>
-      <c r="G15" s="56">
+      <c r="G15" s="57">
         <f>(1.35+1.5+1.65)/3</f>
         <v>1.5</v>
       </c>
-      <c r="H15" s="56">
+      <c r="H15" s="57">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="I15" s="56">
+      <c r="I15" s="57">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="52">
+      <c r="A16" s="53">
         <v>7</v>
       </c>
-      <c r="B16" s="53" t="s">
+      <c r="B16" s="54" t="s">
         <v>80</v>
       </c>
-      <c r="C16" s="54" t="s">
+      <c r="C16" s="55" t="s">
         <v>90</v>
       </c>
-      <c r="D16" s="54" t="s">
+      <c r="D16" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="90">
-        <v>2</v>
-      </c>
-      <c r="F16" s="56">
+      <c r="E16" s="91">
+        <v>2</v>
+      </c>
+      <c r="F16" s="57">
         <f>(2+4.3+5.2)/3</f>
         <v>3.8333333333333335</v>
       </c>
-      <c r="G16" s="56">
+      <c r="G16" s="57">
         <f>(5+6.5+7.2)/3</f>
         <v>6.2333333333333334</v>
       </c>
-      <c r="H16" s="56">
+      <c r="H16" s="57">
         <f t="shared" si="0"/>
         <v>7.666666666666667</v>
       </c>
-      <c r="I16" s="56">
+      <c r="I16" s="57">
         <f t="shared" si="1"/>
         <v>12.466666666666667</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="78">
+      <c r="A17" s="79">
         <v>8</v>
       </c>
-      <c r="B17" s="79" t="s">
+      <c r="B17" s="80" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="80" t="s">
+      <c r="C17" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="80" t="s">
+      <c r="D17" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="92">
-        <v>2</v>
-      </c>
-      <c r="F17" s="82">
+      <c r="E17" s="93">
+        <v>2</v>
+      </c>
+      <c r="F17" s="83">
         <f>(0.72+0.8+0.88)/3</f>
         <v>0.79999999999999993</v>
       </c>
-      <c r="G17" s="82">
+      <c r="G17" s="83">
         <f>(0.72+0.8+0.88)/3</f>
         <v>0.79999999999999993</v>
       </c>
-      <c r="H17" s="82">
+      <c r="H17" s="83">
         <f t="shared" si="0"/>
         <v>1.5999999999999999</v>
       </c>
-      <c r="I17" s="82">
+      <c r="I17" s="83">
         <f t="shared" si="1"/>
         <v>1.5999999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="57">
+      <c r="A18" s="58">
         <v>9</v>
       </c>
-      <c r="B18" s="58" t="s">
+      <c r="B18" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="C18" s="59" t="s">
+      <c r="C18" s="60" t="s">
         <v>93</v>
       </c>
-      <c r="D18" s="59" t="s">
+      <c r="D18" s="60" t="s">
         <v>93</v>
       </c>
-      <c r="E18" s="94">
+      <c r="E18" s="95">
         <v>3</v>
       </c>
-      <c r="F18" s="61">
+      <c r="F18" s="62">
         <f>(16.25+18+19.5)/3</f>
         <v>17.916666666666668</v>
       </c>
-      <c r="G18" s="61">
+      <c r="G18" s="62">
         <f>(16.25+18+19.5)/3</f>
         <v>17.916666666666668</v>
       </c>
-      <c r="H18" s="61">
+      <c r="H18" s="62">
         <f t="shared" si="0"/>
         <v>53.75</v>
       </c>
-      <c r="I18" s="61">
+      <c r="I18" s="62">
         <f t="shared" si="1"/>
         <v>53.75</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="68">
+      <c r="A19" s="69">
         <v>10</v>
       </c>
-      <c r="B19" s="69" t="s">
+      <c r="B19" s="70" t="s">
         <v>80</v>
       </c>
-      <c r="C19" s="70" t="s">
+      <c r="C19" s="71" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="70" t="s">
+      <c r="D19" s="71" t="s">
         <v>94</v>
       </c>
-      <c r="E19" s="96">
-        <v>2</v>
-      </c>
-      <c r="F19" s="72">
+      <c r="E19" s="97">
+        <v>2</v>
+      </c>
+      <c r="F19" s="73">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="G19" s="72">
+      <c r="G19" s="73">
         <f>(1.44+2.3+3.1)/3</f>
         <v>2.2799999999999998</v>
       </c>
-      <c r="H19" s="72">
+      <c r="H19" s="73">
         <f t="shared" si="0"/>
         <v>3.4</v>
       </c>
-      <c r="I19" s="72">
+      <c r="I19" s="73">
         <f t="shared" si="1"/>
         <v>4.5599999999999996</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="68">
+      <c r="A20" s="69">
         <v>10</v>
       </c>
-      <c r="B20" s="69" t="s">
+      <c r="B20" s="70" t="s">
         <v>83</v>
       </c>
-      <c r="C20" s="70" t="s">
+      <c r="C20" s="71" t="s">
         <v>95</v>
       </c>
-      <c r="D20" s="70" t="s">
+      <c r="D20" s="71" t="s">
         <v>96</v>
       </c>
-      <c r="E20" s="96">
+      <c r="E20" s="97">
         <v>3</v>
       </c>
-      <c r="F20" s="72">
+      <c r="F20" s="73">
         <f>(3+4+5)/3</f>
         <v>4</v>
       </c>
-      <c r="G20" s="72">
+      <c r="G20" s="73">
         <f>(3.5+4.5+5.5)/3</f>
         <v>4.5</v>
       </c>
-      <c r="H20" s="72">
+      <c r="H20" s="73">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="I20" s="72">
+      <c r="I20" s="73">
         <f t="shared" si="1"/>
         <v>13.5</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="73">
+      <c r="A21" s="74">
         <v>11</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="B21" s="75" t="s">
         <v>97</v>
       </c>
-      <c r="C21" s="75" t="s">
+      <c r="C21" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="75" t="s">
+      <c r="D21" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="E21" s="76">
+      <c r="E21" s="77">
         <v>1</v>
       </c>
-      <c r="F21" s="77">
+      <c r="F21" s="78">
         <f>(0.45+0.5+0.55)/3</f>
         <v>0.5</v>
       </c>
-      <c r="G21" s="77">
+      <c r="G21" s="78">
         <f>(0.45+0.5+0.55)/3</f>
         <v>0.5</v>
       </c>
-      <c r="H21" s="77">
+      <c r="H21" s="78">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="I21" s="77">
+      <c r="I21" s="78">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
@@ -4064,7 +4061,7 @@
       </c>
       <c r="G22" s="13">
         <f>SUM(G2:G21)</f>
-        <v>90.63333333333334</v>
+        <v>90.213333333333338</v>
       </c>
       <c r="H22" s="13">
         <f>SUM(H3:H21)</f>
@@ -4072,7 +4069,7 @@
       </c>
       <c r="I22" s="13">
         <f>SUM(I3:I21)</f>
-        <v>229.12666666666667</v>
+        <v>228.28666666666666</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4141,7 +4138,7 @@
       </c>
       <c r="D27" s="11">
         <f>MAX(G8)</f>
-        <v>1.8</v>
+        <v>1.3800000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4287,7 +4284,7 @@
       </c>
       <c r="D36" s="13">
         <f>SUM(D25:D35)</f>
-        <v>70.766666666666666</v>
+        <v>70.346666666666664</v>
       </c>
     </row>
   </sheetData>
@@ -4322,10 +4319,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="102" t="s">
+      <c r="B1" s="104" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -4337,22 +4334,22 @@
       <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="101" t="s">
+      <c r="F1" s="103" t="s">
         <v>137</v>
       </c>
-      <c r="G1" s="101" t="s">
+      <c r="G1" s="103" t="s">
         <v>138</v>
       </c>
-      <c r="H1" s="101" t="s">
+      <c r="H1" s="103" t="s">
         <v>153</v>
       </c>
-      <c r="I1" s="101" t="s">
+      <c r="I1" s="103" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="103"/>
-      <c r="B2" s="103"/>
+      <c r="A2" s="105"/>
+      <c r="B2" s="105"/>
       <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
@@ -4362,667 +4359,667 @@
       <c r="E2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="22">
+      <c r="A3" s="23">
         <v>1</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="E3" s="65">
-        <v>2</v>
-      </c>
-      <c r="F3" s="26">
+      <c r="E3" s="66">
+        <v>2</v>
+      </c>
+      <c r="F3" s="27">
         <f>(1.88+2.62+2.82)/3</f>
         <v>2.44</v>
       </c>
-      <c r="G3" s="26">
+      <c r="G3" s="27">
         <f>(1.33+2.25+2.98)/3</f>
         <v>2.186666666666667</v>
       </c>
-      <c r="H3" s="26">
+      <c r="H3" s="27">
         <f>F3*E3</f>
         <v>4.88</v>
       </c>
-      <c r="I3" s="26">
+      <c r="I3" s="27">
         <f>G3*E3</f>
         <v>4.373333333333334</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="22">
+      <c r="A4" s="23">
         <v>1</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="E4" s="65">
+      <c r="E4" s="66">
         <v>4</v>
       </c>
-      <c r="F4" s="26">
+      <c r="F4" s="27">
         <f>(5.2+6.54+7.12)/3</f>
         <v>6.2866666666666662</v>
       </c>
-      <c r="G4" s="26">
+      <c r="G4" s="27">
         <f>(4.2+5.4+6.23)/3</f>
         <v>5.2766666666666673</v>
       </c>
-      <c r="H4" s="26">
+      <c r="H4" s="27">
         <f t="shared" ref="H4:H22" si="0">F4*E4</f>
         <v>25.146666666666665</v>
       </c>
-      <c r="I4" s="26">
+      <c r="I4" s="27">
         <f t="shared" ref="I4:I22" si="1">G4*E4</f>
         <v>21.106666666666669</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27">
-        <v>2</v>
-      </c>
-      <c r="B5" s="28" t="s">
+      <c r="A5" s="28">
+        <v>2</v>
+      </c>
+      <c r="B5" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="67">
-        <v>2</v>
-      </c>
-      <c r="F5" s="31">
+      <c r="E5" s="68">
+        <v>2</v>
+      </c>
+      <c r="F5" s="32">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="G5" s="31">
+      <c r="G5" s="32">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="H5" s="31">
+      <c r="H5" s="32">
         <f t="shared" si="0"/>
         <v>4.5999999999999988</v>
       </c>
-      <c r="I5" s="31">
+      <c r="I5" s="32">
         <f t="shared" si="1"/>
         <v>4.5999999999999988</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="27">
-        <v>2</v>
-      </c>
-      <c r="B6" s="28" t="s">
+      <c r="A6" s="28">
+        <v>2</v>
+      </c>
+      <c r="B6" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="67">
-        <v>2</v>
-      </c>
-      <c r="F6" s="31">
+      <c r="E6" s="68">
+        <v>2</v>
+      </c>
+      <c r="F6" s="32">
         <f>(2.1+2.45+2.58)/3</f>
         <v>2.3766666666666669</v>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="32">
         <f>(2.1+2.45+2.58)/3</f>
         <v>2.3766666666666669</v>
       </c>
-      <c r="H6" s="31">
+      <c r="H6" s="32">
         <f t="shared" si="0"/>
         <v>4.7533333333333339</v>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="32">
         <f t="shared" si="1"/>
         <v>4.7533333333333339</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="32">
+      <c r="A7" s="33">
         <v>3</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="34" t="s">
         <v>104</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="34" t="s">
+      <c r="D7" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="63">
-        <v>2</v>
-      </c>
-      <c r="F7" s="36">
+      <c r="E7" s="64">
+        <v>2</v>
+      </c>
+      <c r="F7" s="37">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="G7" s="36">
+      <c r="G7" s="37">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="H7" s="36">
+      <c r="H7" s="37">
         <f t="shared" si="0"/>
         <v>3.4</v>
       </c>
-      <c r="I7" s="36">
+      <c r="I7" s="37">
         <f t="shared" si="1"/>
         <v>3.4</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="32">
+      <c r="A8" s="33">
         <v>3</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="34" t="s">
         <v>105</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="E8" s="63">
-        <v>2</v>
-      </c>
-      <c r="F8" s="36">
+      <c r="E8" s="64">
+        <v>2</v>
+      </c>
+      <c r="F8" s="37">
         <f>(1.62+1.8+1.98)/3</f>
         <v>1.8</v>
       </c>
-      <c r="G8" s="36">
+      <c r="G8" s="37">
         <f>(1.2+1.34+1.6)/3</f>
         <v>1.3800000000000001</v>
       </c>
-      <c r="H8" s="36">
+      <c r="H8" s="37">
         <f t="shared" si="0"/>
         <v>3.6</v>
       </c>
-      <c r="I8" s="36">
+      <c r="I8" s="37">
         <f t="shared" si="1"/>
         <v>2.7600000000000002</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="32">
+      <c r="A9" s="33">
         <v>3</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="34" t="s">
         <v>106</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="35" t="s">
         <v>107</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="D9" s="35" t="s">
         <v>108</v>
       </c>
-      <c r="E9" s="63">
+      <c r="E9" s="64">
         <v>4</v>
       </c>
-      <c r="F9" s="36">
+      <c r="F9" s="37">
         <f>(18+20+22)/3</f>
         <v>20</v>
       </c>
-      <c r="G9" s="36">
+      <c r="G9" s="37">
         <f>(13.2+15.3+16)/3</f>
         <v>14.833333333333334</v>
       </c>
-      <c r="H9" s="36">
+      <c r="H9" s="37">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="I9" s="36">
+      <c r="I9" s="37">
         <f t="shared" si="1"/>
         <v>59.333333333333336</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="37">
+      <c r="A10" s="38">
         <v>4</v>
       </c>
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="39" t="s">
         <v>109</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="40" t="s">
         <v>110</v>
       </c>
-      <c r="D10" s="39" t="s">
+      <c r="D10" s="40" t="s">
         <v>110</v>
       </c>
-      <c r="E10" s="84">
-        <v>2</v>
-      </c>
-      <c r="F10" s="41">
+      <c r="E10" s="85">
+        <v>2</v>
+      </c>
+      <c r="F10" s="42">
         <f>(1.6+1.8+1.9)/3</f>
         <v>1.7666666666666668</v>
       </c>
-      <c r="G10" s="41">
+      <c r="G10" s="42">
         <f>(1.6+1.8+1.9)/3</f>
         <v>1.7666666666666668</v>
       </c>
-      <c r="H10" s="41">
+      <c r="H10" s="42">
         <f t="shared" si="0"/>
         <v>3.5333333333333337</v>
       </c>
-      <c r="I10" s="41">
+      <c r="I10" s="42">
         <f t="shared" si="1"/>
         <v>3.5333333333333337</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="37">
+      <c r="A11" s="38">
         <v>4</v>
       </c>
-      <c r="B11" s="38" t="s">
+      <c r="B11" s="39" t="s">
         <v>111</v>
       </c>
-      <c r="C11" s="39" t="s">
+      <c r="C11" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="D11" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="84">
-        <v>2</v>
-      </c>
-      <c r="F11" s="41">
+      <c r="E11" s="85">
+        <v>2</v>
+      </c>
+      <c r="F11" s="42">
         <f>(1.89+2.1+2.31)/3</f>
         <v>2.1</v>
       </c>
-      <c r="G11" s="41">
+      <c r="G11" s="42">
         <f>(1.89+2.1+2.31)/3</f>
         <v>2.1</v>
       </c>
-      <c r="H11" s="41">
+      <c r="H11" s="42">
         <f t="shared" si="0"/>
         <v>4.2</v>
       </c>
-      <c r="I11" s="41">
+      <c r="I11" s="42">
         <f t="shared" si="1"/>
         <v>4.2</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="42">
+      <c r="A12" s="43">
         <v>5</v>
       </c>
-      <c r="B12" s="43" t="s">
+      <c r="B12" s="44" t="s">
         <v>112</v>
       </c>
-      <c r="C12" s="44" t="s">
+      <c r="C12" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="44" t="s">
+      <c r="D12" s="45" t="s">
         <v>85</v>
       </c>
-      <c r="E12" s="86">
-        <v>2</v>
-      </c>
-      <c r="F12" s="46">
+      <c r="E12" s="87">
+        <v>2</v>
+      </c>
+      <c r="F12" s="47">
         <f>(2.34+2.6+2.86)/3</f>
         <v>2.5999999999999996</v>
       </c>
-      <c r="G12" s="46">
+      <c r="G12" s="47">
         <f>(2.44+2.65+3.6)/3</f>
         <v>2.8966666666666665</v>
       </c>
-      <c r="H12" s="46">
+      <c r="H12" s="47">
         <f t="shared" si="0"/>
         <v>5.1999999999999993</v>
       </c>
-      <c r="I12" s="46">
+      <c r="I12" s="47">
         <f t="shared" si="1"/>
         <v>5.793333333333333</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="47">
+      <c r="A13" s="48">
         <v>6</v>
       </c>
-      <c r="B13" s="48" t="s">
+      <c r="B13" s="49" t="s">
         <v>113</v>
       </c>
-      <c r="C13" s="49" t="s">
+      <c r="C13" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="D13" s="49" t="s">
+      <c r="D13" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="E13" s="88">
-        <v>2</v>
-      </c>
-      <c r="F13" s="51">
+      <c r="E13" s="89">
+        <v>2</v>
+      </c>
+      <c r="F13" s="52">
         <f>(0.9+1+1.1)/3</f>
         <v>1</v>
       </c>
-      <c r="G13" s="51">
+      <c r="G13" s="52">
         <f>(0.9+1+1.1)/3</f>
         <v>1</v>
       </c>
-      <c r="H13" s="51">
+      <c r="H13" s="52">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="I13" s="51">
+      <c r="I13" s="52">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="47">
+      <c r="A14" s="48">
         <v>6</v>
       </c>
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="49" t="s">
         <v>114</v>
       </c>
-      <c r="C14" s="49" t="s">
+      <c r="C14" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="D14" s="49" t="s">
+      <c r="D14" s="50" t="s">
         <v>88</v>
       </c>
-      <c r="E14" s="88">
+      <c r="E14" s="89">
         <v>3</v>
       </c>
-      <c r="F14" s="51">
+      <c r="F14" s="52">
         <f>(12+15+17)/3</f>
         <v>14.666666666666666</v>
       </c>
-      <c r="G14" s="51">
+      <c r="G14" s="52">
         <f>(10+12+15)/3</f>
         <v>12.333333333333334</v>
       </c>
-      <c r="H14" s="51">
+      <c r="H14" s="52">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="I14" s="51">
+      <c r="I14" s="52">
         <f t="shared" si="1"/>
         <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="47">
+      <c r="A15" s="48">
         <v>6</v>
       </c>
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="49" t="s">
         <v>115</v>
       </c>
-      <c r="C15" s="49" t="s">
+      <c r="C15" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="49" t="s">
+      <c r="D15" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="88">
-        <v>2</v>
-      </c>
-      <c r="F15" s="51">
+      <c r="E15" s="89">
+        <v>2</v>
+      </c>
+      <c r="F15" s="52">
         <f>(1.35+1.5+1.65)/3</f>
         <v>1.5</v>
       </c>
-      <c r="G15" s="51">
+      <c r="G15" s="52">
         <f>(1.35+1.5+1.65)/3</f>
         <v>1.5</v>
       </c>
-      <c r="H15" s="51">
+      <c r="H15" s="52">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="I15" s="51">
+      <c r="I15" s="52">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="52">
+      <c r="A16" s="53">
         <v>7</v>
       </c>
-      <c r="B16" s="53" t="s">
+      <c r="B16" s="54" t="s">
         <v>116</v>
       </c>
-      <c r="C16" s="54" t="s">
+      <c r="C16" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="54" t="s">
+      <c r="D16" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="90">
+      <c r="E16" s="91">
         <v>4</v>
       </c>
-      <c r="F16" s="56">
+      <c r="F16" s="57">
         <f>(5+6.5+7.2)/3</f>
         <v>6.2333333333333334</v>
       </c>
-      <c r="G16" s="56">
+      <c r="G16" s="57">
         <f>(5+6.5+7.2)/3</f>
         <v>6.2333333333333334</v>
       </c>
-      <c r="H16" s="56">
+      <c r="H16" s="57">
         <f t="shared" si="0"/>
         <v>24.933333333333334</v>
       </c>
-      <c r="I16" s="56">
+      <c r="I16" s="57">
         <f t="shared" si="1"/>
         <v>24.933333333333334</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="78">
+      <c r="A17" s="79">
         <v>8</v>
       </c>
-      <c r="B17" s="79" t="s">
+      <c r="B17" s="80" t="s">
         <v>117</v>
       </c>
-      <c r="C17" s="80" t="s">
+      <c r="C17" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="80" t="s">
+      <c r="D17" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="92">
-        <v>2</v>
-      </c>
-      <c r="F17" s="82">
+      <c r="E17" s="93">
+        <v>2</v>
+      </c>
+      <c r="F17" s="83">
         <f>(0.72+0.8+0.88)/3</f>
         <v>0.79999999999999993</v>
       </c>
-      <c r="G17" s="82">
+      <c r="G17" s="83">
         <f>(0.72+0.8+0.88)/3</f>
         <v>0.79999999999999993</v>
       </c>
-      <c r="H17" s="82">
+      <c r="H17" s="83">
         <f t="shared" si="0"/>
         <v>1.5999999999999999</v>
       </c>
-      <c r="I17" s="82">
+      <c r="I17" s="83">
         <f t="shared" si="1"/>
         <v>1.5999999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="57">
+      <c r="A18" s="58">
         <v>9</v>
       </c>
-      <c r="B18" s="58" t="s">
+      <c r="B18" s="59" t="s">
         <v>118</v>
       </c>
-      <c r="C18" s="59" t="s">
+      <c r="C18" s="60" t="s">
         <v>93</v>
       </c>
-      <c r="D18" s="59" t="s">
+      <c r="D18" s="60" t="s">
         <v>93</v>
       </c>
-      <c r="E18" s="94">
+      <c r="E18" s="95">
         <v>4</v>
       </c>
-      <c r="F18" s="61">
+      <c r="F18" s="62">
         <f>(16.25+18+19.5)/3</f>
         <v>17.916666666666668</v>
       </c>
-      <c r="G18" s="61">
+      <c r="G18" s="62">
         <f>(16.25+18+19.5)/3</f>
         <v>17.916666666666668</v>
       </c>
-      <c r="H18" s="61">
+      <c r="H18" s="62">
         <f t="shared" si="0"/>
         <v>71.666666666666671</v>
       </c>
-      <c r="I18" s="61">
+      <c r="I18" s="62">
         <f t="shared" si="1"/>
         <v>71.666666666666671</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="57">
+      <c r="A19" s="58">
         <v>9</v>
       </c>
-      <c r="B19" s="58" t="s">
+      <c r="B19" s="59" t="s">
         <v>119</v>
       </c>
-      <c r="C19" s="59" t="s">
+      <c r="C19" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="59" t="s">
+      <c r="D19" s="60" t="s">
         <v>94</v>
       </c>
-      <c r="E19" s="94">
-        <v>2</v>
-      </c>
-      <c r="F19" s="61">
+      <c r="E19" s="95">
+        <v>2</v>
+      </c>
+      <c r="F19" s="62">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="G19" s="61">
+      <c r="G19" s="62">
         <f>(1.44+2.3+3.1)/3</f>
         <v>2.2799999999999998</v>
       </c>
-      <c r="H19" s="61">
+      <c r="H19" s="62">
         <f t="shared" si="0"/>
         <v>3.4</v>
       </c>
-      <c r="I19" s="61">
+      <c r="I19" s="62">
         <f t="shared" si="1"/>
         <v>4.5599999999999996</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="68">
+      <c r="A20" s="69">
         <v>10</v>
       </c>
-      <c r="B20" s="69" t="s">
+      <c r="B20" s="70" t="s">
         <v>120</v>
       </c>
-      <c r="C20" s="70" t="s">
+      <c r="C20" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="D20" s="70" t="s">
+      <c r="D20" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="E20" s="96">
+      <c r="E20" s="97">
         <v>3</v>
       </c>
-      <c r="F20" s="72">
+      <c r="F20" s="73">
         <f>(0.9+1+1.1)/3</f>
         <v>1</v>
       </c>
-      <c r="G20" s="72">
+      <c r="G20" s="73">
         <f>(0.9+1+1.1)/3</f>
         <v>1</v>
       </c>
-      <c r="H20" s="72">
+      <c r="H20" s="73">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="I20" s="72">
+      <c r="I20" s="73">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="73">
+      <c r="A21" s="74">
         <v>11</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="B21" s="75" t="s">
         <v>121</v>
       </c>
-      <c r="C21" s="75" t="s">
+      <c r="C21" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="75" t="s">
+      <c r="D21" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="E21" s="98">
+      <c r="E21" s="99">
         <v>1</v>
       </c>
-      <c r="F21" s="77">
+      <c r="F21" s="78">
         <f>(0.45+0.5+0.55)/3</f>
         <v>0.5</v>
       </c>
-      <c r="G21" s="77">
+      <c r="G21" s="78">
         <f>(0.45+0.5+0.55)/3</f>
         <v>0.5</v>
       </c>
-      <c r="H21" s="77">
+      <c r="H21" s="78">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="I21" s="77">
+      <c r="I21" s="78">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="73">
+      <c r="A22" s="74">
         <v>11</v>
       </c>
-      <c r="B22" s="74" t="s">
+      <c r="B22" s="75" t="s">
         <v>122</v>
       </c>
-      <c r="C22" s="75" t="s">
+      <c r="C22" s="76" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="75" t="s">
+      <c r="D22" s="76" t="s">
         <v>29</v>
       </c>
-      <c r="E22" s="98">
+      <c r="E22" s="99">
         <v>3</v>
       </c>
-      <c r="F22" s="77">
+      <c r="F22" s="78">
         <f>(1.71+1.9+2.09)/3</f>
         <v>1.8999999999999997</v>
       </c>
-      <c r="G22" s="77">
+      <c r="G22" s="78">
         <f>(1.71+1.9+2.09)/3</f>
         <v>1.8999999999999997</v>
       </c>
-      <c r="H22" s="77">
+      <c r="H22" s="78">
         <f t="shared" si="0"/>
         <v>5.6999999999999993</v>
       </c>
-      <c r="I22" s="77">
+      <c r="I22" s="78">
         <f t="shared" si="1"/>
         <v>5.6999999999999993</v>
       </c>
@@ -5284,10 +5281,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="102" t="s">
+      <c r="B1" s="104" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -5299,22 +5296,22 @@
       <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="101" t="s">
+      <c r="F1" s="103" t="s">
         <v>137</v>
       </c>
-      <c r="G1" s="101" t="s">
+      <c r="G1" s="103" t="s">
         <v>138</v>
       </c>
-      <c r="H1" s="101" t="s">
+      <c r="H1" s="103" t="s">
         <v>153</v>
       </c>
-      <c r="I1" s="101" t="s">
+      <c r="I1" s="103" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="103"/>
-      <c r="B2" s="103"/>
+      <c r="A2" s="105"/>
+      <c r="B2" s="105"/>
       <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
@@ -5324,172 +5321,172 @@
       <c r="E2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="22">
+      <c r="A3" s="23">
         <v>1</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="65">
-        <v>2</v>
-      </c>
-      <c r="F3" s="26">
+      <c r="E3" s="66">
+        <v>2</v>
+      </c>
+      <c r="F3" s="27">
         <f>(1.98+2.2+2.42)/3</f>
         <v>2.1999999999999997</v>
       </c>
-      <c r="G3" s="26">
+      <c r="G3" s="27">
         <f>(1.98+2.2+2.42)/3</f>
         <v>2.1999999999999997</v>
       </c>
-      <c r="H3" s="26">
+      <c r="H3" s="27">
         <f>F3*E3</f>
         <v>4.3999999999999995</v>
       </c>
-      <c r="I3" s="26">
+      <c r="I3" s="27">
         <f>G3*E3</f>
         <v>4.3999999999999995</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="22">
+      <c r="A4" s="23">
         <v>1</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="24" t="s">
         <v>124</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="65">
+      <c r="E4" s="66">
         <v>3</v>
       </c>
-      <c r="F4" s="26">
+      <c r="F4" s="27">
         <f>(1.98+2.2+2.42)/3</f>
         <v>2.1999999999999997</v>
       </c>
-      <c r="G4" s="26">
+      <c r="G4" s="27">
         <f>(1.98+2.2+2.42)/3</f>
         <v>2.1999999999999997</v>
       </c>
-      <c r="H4" s="26">
+      <c r="H4" s="27">
         <f t="shared" ref="H4:H7" si="0">F4*E4</f>
         <v>6.6</v>
       </c>
-      <c r="I4" s="26">
+      <c r="I4" s="27">
         <f t="shared" ref="I4:I7" si="1">G4*E4</f>
         <v>6.6</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27">
-        <v>2</v>
-      </c>
-      <c r="B5" s="28" t="s">
+      <c r="A5" s="28">
+        <v>2</v>
+      </c>
+      <c r="B5" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="67">
-        <v>2</v>
-      </c>
-      <c r="F5" s="31">
+      <c r="E5" s="68">
+        <v>2</v>
+      </c>
+      <c r="F5" s="32">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="G5" s="31">
+      <c r="G5" s="32">
         <f>(2.07+2.3+2.53)/3</f>
         <v>2.2999999999999994</v>
       </c>
-      <c r="H5" s="31">
+      <c r="H5" s="32">
         <f t="shared" si="0"/>
         <v>4.5999999999999988</v>
       </c>
-      <c r="I5" s="31">
+      <c r="I5" s="32">
         <f t="shared" si="1"/>
         <v>4.5999999999999988</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="27">
-        <v>2</v>
-      </c>
-      <c r="B6" s="28" t="s">
+      <c r="A6" s="28">
+        <v>2</v>
+      </c>
+      <c r="B6" s="29" t="s">
         <v>126</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="30" t="s">
         <v>127</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="30" t="s">
         <v>127</v>
       </c>
-      <c r="E6" s="67">
-        <v>2</v>
-      </c>
-      <c r="F6" s="31">
+      <c r="E6" s="68">
+        <v>2</v>
+      </c>
+      <c r="F6" s="32">
         <f>(2.25+2.5+2.75)/3</f>
         <v>2.5</v>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="32">
         <f>(2.25+2.5+2.75)/3</f>
         <v>2.5</v>
       </c>
-      <c r="H6" s="31">
+      <c r="H6" s="32">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="32">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="32">
+      <c r="A7" s="33">
         <v>3</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="34" t="s">
         <v>128</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="34" t="s">
+      <c r="D7" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="63">
-        <v>2</v>
-      </c>
-      <c r="F7" s="36">
+      <c r="E7" s="64">
+        <v>2</v>
+      </c>
+      <c r="F7" s="37">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="G7" s="36">
+      <c r="G7" s="37">
         <f>(1.53+1.7+1.87)/3</f>
         <v>1.7</v>
       </c>
-      <c r="H7" s="36">
+      <c r="H7" s="37">
         <f t="shared" si="0"/>
         <v>3.4</v>
       </c>
-      <c r="I7" s="36">
+      <c r="I7" s="37">
         <f t="shared" si="1"/>
         <v>3.4</v>
       </c>
@@ -5535,12 +5532,12 @@
         <v>5</v>
       </c>
       <c r="C12" s="11">
-        <f>MAX(H3:H4)</f>
-        <v>6.6</v>
+        <f>MAX(F3:F4)</f>
+        <v>2.1999999999999997</v>
       </c>
       <c r="D12" s="11">
-        <f>MAX(I3:I4)</f>
-        <v>6.6</v>
+        <f>MAX(G3:G4)</f>
+        <v>2.1999999999999997</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -5552,12 +5549,12 @@
         <v>4</v>
       </c>
       <c r="C13" s="11">
-        <f>MAX(H5:H6)</f>
-        <v>5</v>
+        <f>MAX(F5:F6)</f>
+        <v>2.5</v>
       </c>
       <c r="D13" s="11">
-        <f>MAX(I5:I6)</f>
-        <v>5</v>
+        <f>MAX(G5:G6)</f>
+        <v>2.5</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -5569,22 +5566,22 @@
         <v>2</v>
       </c>
       <c r="C14" s="11">
-        <f>MAX(H7)</f>
-        <v>3.4</v>
+        <f>MAX(F7)</f>
+        <v>1.7</v>
       </c>
       <c r="D14" s="11">
-        <f>MAX(I7)</f>
-        <v>3.4</v>
+        <f>MAX(G7)</f>
+        <v>1.7</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C15" s="13">
         <f>SUM(C12:C14)</f>
-        <v>15</v>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D15" s="13">
         <f>SUM(D12:D14)</f>
-        <v>15</v>
+        <v>6.3999999999999995</v>
       </c>
     </row>
   </sheetData>
@@ -5605,7 +5602,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{450BF008-BB3E-4CC7-A7EA-6413059DDDCB}">
-  <dimension ref="A1:U30"/>
+  <dimension ref="A1:U29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -5656,24 +5653,24 @@
         <f t="shared" ref="D3:D6" si="0">SUM(B3:C3)</f>
         <v>233.29000000000002</v>
       </c>
-      <c r="F3" s="104" t="s">
+      <c r="F3" s="106" t="s">
         <v>151</v>
       </c>
-      <c r="G3" s="104"/>
-      <c r="H3" s="104"/>
-      <c r="I3" s="104"/>
-      <c r="J3" s="104"/>
-      <c r="K3" s="104"/>
-      <c r="L3" s="104"/>
-      <c r="M3" s="104"/>
-      <c r="N3" s="104"/>
-      <c r="O3" s="104"/>
-      <c r="P3" s="104"/>
-      <c r="Q3" s="104"/>
-      <c r="R3" s="104"/>
-      <c r="S3" s="104"/>
-      <c r="T3" s="104"/>
-      <c r="U3" s="104"/>
+      <c r="G3" s="106"/>
+      <c r="H3" s="106"/>
+      <c r="I3" s="106"/>
+      <c r="J3" s="106"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="106"/>
+      <c r="M3" s="106"/>
+      <c r="N3" s="106"/>
+      <c r="O3" s="106"/>
+      <c r="P3" s="106"/>
+      <c r="Q3" s="106"/>
+      <c r="R3" s="106"/>
+      <c r="S3" s="106"/>
+      <c r="T3" s="106"/>
+      <c r="U3" s="106"/>
     </row>
     <row r="4" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
@@ -5683,14 +5680,14 @@
         <v>87.15</v>
       </c>
       <c r="C4" s="11">
-        <v>90.633300000000006</v>
+        <v>90.213300000000004</v>
       </c>
       <c r="D4" s="11">
         <f t="shared" si="0"/>
-        <v>177.7833</v>
+        <v>177.36330000000001</v>
       </c>
       <c r="F4" s="19">
-        <v>779.92330000000004</v>
+        <v>779.50329999999997</v>
       </c>
     </row>
     <row r="5" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5736,11 +5733,11 @@
       </c>
       <c r="C7" s="11">
         <f>SUM(C2:C6)</f>
-        <v>380.31999999999994</v>
+        <v>379.9</v>
       </c>
       <c r="D7" s="20">
         <f>SUM(B7:C7)</f>
-        <v>779.92329999999993</v>
+        <v>779.50329999999997</v>
       </c>
       <c r="F7" t="s">
         <v>152</v>
@@ -5749,7 +5746,7 @@
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="D8" s="18"/>
       <c r="F8" s="19">
-        <v>2185.3833</v>
+        <v>2184.5432999999998</v>
       </c>
     </row>
     <row r="9" spans="1:21" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5807,11 +5804,11 @@
         <v>224.35</v>
       </c>
       <c r="C12" s="11">
-        <v>229.1267</v>
+        <v>228.2867</v>
       </c>
       <c r="D12" s="11">
         <f t="shared" si="1"/>
-        <v>453.47669999999999</v>
+        <v>452.63670000000002</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5832,7 +5829,7 @@
         <v>160</v>
       </c>
       <c r="I13" s="19">
-        <v>341.19659999999999</v>
+        <v>332.59660000000002</v>
       </c>
       <c r="J13" t="s">
         <v>162</v>
@@ -5856,7 +5853,7 @@
         <v>161</v>
       </c>
       <c r="I14" s="19">
-        <v>319.58339999999998</v>
+        <v>310.5634</v>
       </c>
       <c r="J14" t="s">
         <v>162</v>
@@ -5872,11 +5869,11 @@
       </c>
       <c r="C15" s="11">
         <f>SUM(C10:C14)</f>
-        <v>1059.0867000000001</v>
+        <v>1058.2467000000001</v>
       </c>
       <c r="D15" s="20">
         <f>SUM(B15:C15)</f>
-        <v>2185.3833000000004</v>
+        <v>2184.5433000000003</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
@@ -5904,7 +5901,7 @@
         <v>177</v>
       </c>
       <c r="K17" s="19"/>
-      <c r="L17" s="100"/>
+      <c r="L17" s="102"/>
     </row>
     <row r="18" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
@@ -5924,7 +5921,7 @@
         <v>178</v>
       </c>
       <c r="K18" s="19"/>
-      <c r="L18" s="100"/>
+      <c r="L18" s="102"/>
     </row>
     <row r="19" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
@@ -5947,7 +5944,7 @@
         <v>181</v>
       </c>
       <c r="K19" s="19"/>
-      <c r="L19" s="100"/>
+      <c r="L19" s="102"/>
     </row>
     <row r="20" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
@@ -5957,17 +5954,17 @@
         <v>67.849999999999994</v>
       </c>
       <c r="C20" s="11">
-        <v>70.7667</v>
+        <v>70.346699999999998</v>
       </c>
       <c r="D20" s="11">
         <f t="shared" si="2"/>
-        <v>138.61669999999998</v>
+        <v>138.19669999999999</v>
       </c>
       <c r="J20" s="19" t="s">
         <v>180</v>
       </c>
       <c r="K20" s="19"/>
-      <c r="L20" s="100"/>
+      <c r="L20" s="102"/>
     </row>
     <row r="21" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
@@ -5989,14 +5986,14 @@
         <v>143</v>
       </c>
       <c r="B22" s="11">
-        <v>15</v>
+        <v>6.4</v>
       </c>
       <c r="C22" s="11">
-        <v>15</v>
+        <v>6.4</v>
       </c>
       <c r="D22" s="11">
         <f t="shared" si="2"/>
-        <v>30</v>
+        <v>12.8</v>
       </c>
       <c r="M22" t="s">
         <v>174</v>
@@ -6008,198 +6005,186 @@
       </c>
       <c r="B23" s="11">
         <f>SUM(B18:B22)</f>
-        <v>341.19659999999999</v>
+        <v>332.59659999999997</v>
       </c>
       <c r="C23" s="11">
         <f>SUM(C18:C22)</f>
-        <v>319.58339999999998</v>
+        <v>310.5634</v>
       </c>
       <c r="D23" s="20">
         <f>SUM(B23:C23)</f>
-        <v>660.78</v>
+        <v>643.16</v>
       </c>
       <c r="M23" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" s="9"/>
-      <c r="B25" s="9" t="s">
+      <c r="B25" t="s">
         <v>167</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" t="s">
         <v>168</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" t="s">
         <v>169</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" t="s">
         <v>170</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="F25" t="s">
         <v>171</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" t="s">
         <v>172</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="H25" t="s">
         <v>173</v>
       </c>
-      <c r="I25" s="9" t="s">
+      <c r="I25" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A26" s="105" t="s">
+      <c r="A26" s="17" t="s">
         <v>163</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26">
         <v>8</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26">
         <v>8</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26">
         <f>B26*C26</f>
         <v>64</v>
       </c>
-      <c r="E26" s="9">
+      <c r="E26">
         <f>B26*C26</f>
         <v>64</v>
       </c>
-      <c r="F26" s="9">
+      <c r="F26">
         <f>B26*C26</f>
         <v>64</v>
       </c>
-      <c r="G26" s="9">
+      <c r="G26">
         <f>B26*C26</f>
         <v>64</v>
       </c>
-      <c r="H26" s="9">
+      <c r="H26">
         <f>B26*C26</f>
         <v>64</v>
       </c>
-      <c r="I26" s="9">
+      <c r="I26">
         <f>SUM(D26:H26)</f>
         <v>320</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A27" s="105" t="s">
+      <c r="A27" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27">
         <v>7</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27">
         <v>8</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27">
         <f t="shared" ref="D27:D29" si="3">B27*C27</f>
         <v>56</v>
       </c>
-      <c r="E27" s="9">
+      <c r="E27">
         <f t="shared" ref="E27:E29" si="4">B27*C27</f>
         <v>56</v>
       </c>
-      <c r="F27" s="9">
+      <c r="F27">
         <f t="shared" ref="F27:F29" si="5">B27*C27</f>
         <v>56</v>
       </c>
-      <c r="G27" s="9">
+      <c r="G27">
         <f t="shared" ref="G27:G29" si="6">B27*C27</f>
         <v>56</v>
       </c>
-      <c r="H27" s="9">
+      <c r="H27">
         <f t="shared" ref="H27:H29" si="7">B27*C27</f>
         <v>56</v>
       </c>
-      <c r="I27" s="9">
+      <c r="I27">
         <f t="shared" ref="I27:I29" si="8">SUM(D27:H27)</f>
         <v>280</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" s="105" t="s">
+      <c r="A28" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28">
         <v>15</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28">
         <v>8</v>
       </c>
-      <c r="D28" s="106">
+      <c r="D28" s="101">
         <f t="shared" si="3"/>
         <v>120</v>
       </c>
-      <c r="E28" s="106">
+      <c r="E28" s="101">
         <f t="shared" si="4"/>
         <v>120</v>
       </c>
-      <c r="F28" s="106">
+      <c r="F28" s="101">
         <f t="shared" si="5"/>
         <v>120</v>
       </c>
-      <c r="G28" s="106">
+      <c r="G28" s="101">
         <f t="shared" si="6"/>
         <v>120</v>
       </c>
-      <c r="H28" s="106">
+      <c r="H28" s="101">
         <f t="shared" si="7"/>
         <v>120</v>
       </c>
-      <c r="I28" s="107">
+      <c r="I28" s="22">
         <f t="shared" si="8"/>
         <v>600</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" s="105" t="s">
+      <c r="A29" s="17" t="s">
         <v>166</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29">
         <f>B28*5</f>
         <v>75</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29">
         <v>8</v>
       </c>
-      <c r="D29" s="106">
+      <c r="D29" s="101">
         <f t="shared" si="3"/>
         <v>600</v>
       </c>
-      <c r="E29" s="106">
+      <c r="E29" s="101">
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="F29" s="106">
+      <c r="F29" s="101">
         <f t="shared" si="5"/>
         <v>600</v>
       </c>
-      <c r="G29" s="106">
+      <c r="G29" s="101">
         <f t="shared" si="6"/>
         <v>600</v>
       </c>
-      <c r="H29" s="106">
+      <c r="H29" s="101">
         <f t="shared" si="7"/>
         <v>600</v>
       </c>
-      <c r="I29" s="107">
+      <c r="I29" s="22">
         <f t="shared" si="8"/>
         <v>3000</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A30" s="9"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>